<commit_message>
set auto dissoc to Y for first row in example
</commit_message>
<xml_diff>
--- a/inst/extdata/sample_sheet.xlsx
+++ b/inst/extdata/sample_sheet.xlsx
@@ -831,7 +831,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:S168"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.35"/>
@@ -963,7 +963,7 @@
         <v>26</v>
       </c>
       <c r="R2" s="0" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="S2" s="0" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
smaller data files for CRAN, updated so that entire data does not need to be imported
</commit_message>
<xml_diff>
--- a/inst/extdata/sample_sheet.xlsx
+++ b/inst/extdata/sample_sheet.xlsx
@@ -831,7 +831,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:S168"/>
-  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.35"/>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>3</v>
@@ -1266,7 +1266,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>28</v>
@@ -1443,7 +1443,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
specify concentrations in example for ROI's 1,2,3
</commit_message>
<xml_diff>
--- a/inst/extdata/sample_sheet.xlsx
+++ b/inst/extdata/sample_sheet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="37">
   <si>
     <t xml:space="preserve">Incl.</t>
   </si>
@@ -97,43 +97,40 @@
     <t xml:space="preserve">7.14E-10, 1.43E-09, 2.86E-09, 5.71E-09, 1.14E-08, 2.28E-08, 4.57E-08, 9.14E-08, 1.83E-07, 3.66E-07, 7.31E-07, 1.46E-06, 2.92E-06</t>
   </si>
   <si>
+    <t xml:space="preserve">2.86E-09, 5.71E-09, 1.14E-08, 2.28E-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antibody001 low conc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.43E-09, 2.86E-09, 5.71E-09, 1.14E-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antibody002 low conc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antibody003 low conc</t>
+  </si>
+  <si>
     <t xml:space="preserve">All</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Antibody001 low conc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.43E-09, 2.86E-09, 5.71E-09, 1.14E-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Antibody002 low conc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.86E-09, 5.71E-09, 1.14E-08, 2.28E-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Antibody003 low conc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.43E-09, 2.86E-09, 5.71E-09, 1.14E-08, 2.28E-08</t>
   </si>
 </sst>
 </file>
@@ -143,7 +140,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -164,6 +161,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -208,12 +210,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -348,7 +354,7 @@
       <c r="K2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="M2" s="1" t="s">
@@ -467,7 +473,7 @@
         <v>24</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>26</v>
@@ -526,7 +532,7 @@
         <v>24</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>26</v>
@@ -558,13 +564,13 @@
         <v>31</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>120</v>
@@ -585,7 +591,7 @@
         <v>24</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>26</v>

</xml_diff>